<commit_message>
Solved Q001 - Sum of Two Numbers
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3a8b2d988c5e44ae/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C9DDAD76-D439-4A50-B4CF-0FD6A90B2464}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F68A53-812B-4234-A82A-96AE79256F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="80">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -279,6 +279,21 @@
   </si>
   <si>
     <t>Remarks</t>
+  </si>
+  <si>
+    <t>Sum of Two Numbers</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>2 mins</t>
+  </si>
+  <si>
+    <t>Learned Scanner &amp; Output</t>
   </si>
 </sst>
 </file>
@@ -343,15 +358,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -673,14 +689,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -758,19 +774,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>74</v>
       </c>
     </row>
@@ -782,7 +798,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -801,47 +817,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="L1" s="3" t="s">
+      <c r="L1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="N1" s="3" t="s">
+      <c r="N1" s="1" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G2" s="4">
+        <v>46188</v>
+      </c>
+      <c r="H2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="N2" t="s">
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -863,22 +914,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>27</v>
       </c>
     </row>
@@ -901,22 +952,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
@@ -940,22 +991,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1076,13 +1127,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1185,22 +1236,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1223,22 +1274,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1261,19 +1312,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>25</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Solved PB002 - Even Or Odd
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F68A53-812B-4234-A82A-96AE79256F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930652AA-33C4-43DF-A1E6-8B58FC613719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -31,7 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'LeetCode Tracker'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Mistake Log'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Pattern Tracker'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progress Tracker'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Progress Tracker'!$A$1:$K$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Revision tracker'!$A$1:$F$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Topic Progress'!$A$1:$F$1</definedName>
   </definedNames>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="91">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -293,14 +293,47 @@
     <t>2 mins</t>
   </si>
   <si>
-    <t>Learned Scanner &amp; Output</t>
+    <t>Welcome toJava</t>
+  </si>
+  <si>
+    <t>Java Stdin and Stdout I</t>
+  </si>
+  <si>
+    <t>Java If-Else</t>
+  </si>
+  <si>
+    <t>HackerRank</t>
+  </si>
+  <si>
+    <t>1 min</t>
+  </si>
+  <si>
+    <t>1.5 min</t>
+  </si>
+  <si>
+    <t>3 min</t>
+  </si>
+  <si>
+    <t>Basic I/O</t>
+  </si>
+  <si>
+    <t>Basic Input</t>
+  </si>
+  <si>
+    <t>Scanner</t>
+  </si>
+  <si>
+    <t>Conditions</t>
+  </si>
+  <si>
+    <t>Even or Odd</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -331,8 +364,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -342,6 +382,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -358,16 +404,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -689,14 +737,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -798,7 +846,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -848,17 +896,11 @@
         <v>21</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>25</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="3"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A2">
@@ -879,7 +921,7 @@
       <c r="F2" t="s">
         <v>77</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="2">
         <v>46188</v>
       </c>
       <c r="H2" t="s">
@@ -891,12 +933,152 @@
       <c r="J2">
         <v>5</v>
       </c>
-      <c r="N2" t="s">
+      <c r="K2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" t="s">
         <v>79</v>
       </c>
+      <c r="D3" t="s">
+        <v>82</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H3" t="s">
+        <v>83</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>5</v>
+      </c>
+      <c r="K3" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D4" t="s">
+        <v>82</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G4" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H4" t="s">
+        <v>84</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>5</v>
+      </c>
+      <c r="K4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" t="s">
+        <v>81</v>
+      </c>
+      <c r="D5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>77</v>
+      </c>
+      <c r="G5" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H5" t="s">
+        <v>85</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G6" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H6" t="s">
+        <v>85</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>5</v>
+      </c>
+      <c r="K6" t="s">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N1" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}"/>
+  <autoFilter ref="A1:K1" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Solved PB003 – Swap Two Numbers
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930652AA-33C4-43DF-A1E6-8B58FC613719}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54994E92-4BC0-4A33-BBCF-13369C84A568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="94">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -327,6 +327,15 @@
   </si>
   <si>
     <t>Even or Odd</t>
+  </si>
+  <si>
+    <t>Swap Two Numbers</t>
+  </si>
+  <si>
+    <t>3.5 min</t>
+  </si>
+  <si>
+    <t>Variables</t>
   </si>
 </sst>
 </file>
@@ -846,7 +855,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1075,6 +1084,41 @@
       </c>
       <c r="K6" t="s">
         <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D7" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>77</v>
+      </c>
+      <c r="G7" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H7" t="s">
+        <v>92</v>
+      </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
+      <c r="J7">
+        <v>5</v>
+      </c>
+      <c r="K7" t="s">
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB004 Largest of Two Numbers
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54994E92-4BC0-4A33-BBCF-13369C84A568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E469CE0C-34CC-4B8C-AE84-B8DA51269CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="5772" yWindow="372" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="96">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -336,6 +336,12 @@
   </si>
   <si>
     <t>Variables</t>
+  </si>
+  <si>
+    <t>Largest of Two Numbers</t>
+  </si>
+  <si>
+    <t>Operators</t>
   </si>
 </sst>
 </file>
@@ -855,7 +861,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1119,6 +1125,41 @@
       </c>
       <c r="K7" t="s">
         <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>94</v>
+      </c>
+      <c r="D8" t="s">
+        <v>76</v>
+      </c>
+      <c r="E8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" t="s">
+        <v>77</v>
+      </c>
+      <c r="G8" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H8" t="s">
+        <v>85</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>5</v>
+      </c>
+      <c r="K8" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB005 - Largest Of Three Numbers
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E469CE0C-34CC-4B8C-AE84-B8DA51269CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102FF31D-657F-4406-AF3A-2042201FD230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5772" yWindow="372" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="100">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -342,6 +342,18 @@
   </si>
   <si>
     <t>Operators</t>
+  </si>
+  <si>
+    <t>Largest of Three Numbers</t>
+  </si>
+  <si>
+    <t>Java Loops I</t>
+  </si>
+  <si>
+    <t>4 min</t>
+  </si>
+  <si>
+    <t>If-Else</t>
   </si>
 </sst>
 </file>
@@ -861,7 +873,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1160,6 +1172,76 @@
       </c>
       <c r="K8" t="s">
         <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F9" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H9" t="s">
+        <v>98</v>
+      </c>
+      <c r="I9">
+        <v>1</v>
+      </c>
+      <c r="J9">
+        <v>5</v>
+      </c>
+      <c r="K9" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" t="s">
+        <v>77</v>
+      </c>
+      <c r="G10" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H10" t="s">
+        <v>84</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>5</v>
+      </c>
+      <c r="K10" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB006 Positive Negative or Zero
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{102FF31D-657F-4406-AF3A-2042201FD230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD0BB39-5295-4D9F-8544-F2B57CE2C03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="101">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -290,9 +290,6 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>2 mins</t>
-  </si>
-  <si>
     <t>Welcome toJava</t>
   </si>
   <si>
@@ -350,10 +347,16 @@
     <t>Java Loops I</t>
   </si>
   <si>
+    <t>2 min</t>
+  </si>
+  <si>
     <t>4 min</t>
   </si>
   <si>
     <t>If-Else</t>
+  </si>
+  <si>
+    <t>Positive Negative or Zero</t>
   </si>
 </sst>
 </file>
@@ -873,7 +876,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -952,7 +955,7 @@
         <v>46188</v>
       </c>
       <c r="H2" t="s">
-        <v>78</v>
+        <v>97</v>
       </c>
       <c r="I2">
         <v>1</v>
@@ -961,7 +964,7 @@
         <v>5</v>
       </c>
       <c r="K2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -972,10 +975,10 @@
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E3" t="s">
         <v>4</v>
@@ -987,7 +990,7 @@
         <v>46188</v>
       </c>
       <c r="H3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I3">
         <v>1</v>
@@ -996,7 +999,7 @@
         <v>5</v>
       </c>
       <c r="K3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -1007,10 +1010,10 @@
         <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E4" t="s">
         <v>4</v>
@@ -1022,7 +1025,7 @@
         <v>46188</v>
       </c>
       <c r="H4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I4">
         <v>1</v>
@@ -1031,7 +1034,7 @@
         <v>5</v>
       </c>
       <c r="K4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -1042,10 +1045,10 @@
         <v>34</v>
       </c>
       <c r="C5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" t="s">
         <v>81</v>
-      </c>
-      <c r="D5" t="s">
-        <v>82</v>
       </c>
       <c r="E5" t="s">
         <v>4</v>
@@ -1057,7 +1060,7 @@
         <v>46188</v>
       </c>
       <c r="H5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I5">
         <v>1</v>
@@ -1066,7 +1069,7 @@
         <v>5</v>
       </c>
       <c r="K5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -1077,7 +1080,7 @@
         <v>34</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D6" t="s">
         <v>76</v>
@@ -1092,7 +1095,7 @@
         <v>46188</v>
       </c>
       <c r="H6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I6">
         <v>1</v>
@@ -1101,7 +1104,7 @@
         <v>5</v>
       </c>
       <c r="K6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -1112,7 +1115,7 @@
         <v>34</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D7" t="s">
         <v>76</v>
@@ -1127,7 +1130,7 @@
         <v>46188</v>
       </c>
       <c r="H7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="I7">
         <v>1</v>
@@ -1136,7 +1139,7 @@
         <v>5</v>
       </c>
       <c r="K7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -1147,7 +1150,7 @@
         <v>34</v>
       </c>
       <c r="C8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D8" t="s">
         <v>76</v>
@@ -1162,7 +1165,7 @@
         <v>46188</v>
       </c>
       <c r="H8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I8">
         <v>1</v>
@@ -1171,7 +1174,7 @@
         <v>5</v>
       </c>
       <c r="K8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1182,7 +1185,7 @@
         <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D9" t="s">
         <v>76</v>
@@ -1217,10 +1220,10 @@
         <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E10" t="s">
         <v>4</v>
@@ -1232,7 +1235,7 @@
         <v>46189</v>
       </c>
       <c r="H10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I10">
         <v>1</v>
@@ -1241,6 +1244,41 @@
         <v>5</v>
       </c>
       <c r="K10" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" t="s">
+        <v>100</v>
+      </c>
+      <c r="D11" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" t="s">
+        <v>4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>77</v>
+      </c>
+      <c r="G11" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H11" t="s">
+        <v>97</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>5</v>
+      </c>
+      <c r="K11" t="s">
         <v>99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Solved PB007 Leap Year
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BD0BB39-5295-4D9F-8544-F2B57CE2C03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FF4BC8-4C22-481A-9E58-D56403519A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="105">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -357,6 +357,18 @@
   </si>
   <si>
     <t>Positive Negative or Zero</t>
+  </si>
+  <si>
+    <t>Leap Year</t>
+  </si>
+  <si>
+    <t>16=06-2026</t>
+  </si>
+  <si>
+    <t>5 min</t>
+  </si>
+  <si>
+    <t>Conditions, If-Else</t>
   </si>
 </sst>
 </file>
@@ -876,7 +888,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1280,6 +1292,41 @@
       </c>
       <c r="K11" t="s">
         <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D12" t="s">
+        <v>76</v>
+      </c>
+      <c r="E12" t="s">
+        <v>4</v>
+      </c>
+      <c r="F12" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" t="s">
+        <v>102</v>
+      </c>
+      <c r="H12" t="s">
+        <v>103</v>
+      </c>
+      <c r="I12">
+        <v>2</v>
+      </c>
+      <c r="J12">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="K12" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB008 Multiplication Table
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FF4BC8-4C22-481A-9E58-D56403519A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC499C6-A34C-4683-B5EF-7E166C102D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="107">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -362,13 +362,19 @@
     <t>Leap Year</t>
   </si>
   <si>
-    <t>16=06-2026</t>
-  </si>
-  <si>
     <t>5 min</t>
   </si>
   <si>
     <t>Conditions, If-Else</t>
+  </si>
+  <si>
+    <t>Multiplication Table</t>
+  </si>
+  <si>
+    <t>Loops</t>
+  </si>
+  <si>
+    <t>Loops, If-Else</t>
   </si>
 </sst>
 </file>
@@ -888,7 +894,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N12"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1256,7 +1262,7 @@
         <v>5</v>
       </c>
       <c r="K10" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.3">
@@ -1313,11 +1319,11 @@
       <c r="F12" t="s">
         <v>77</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H12" t="s">
         <v>102</v>
-      </c>
-      <c r="H12" t="s">
-        <v>103</v>
       </c>
       <c r="I12">
         <v>2</v>
@@ -1326,7 +1332,47 @@
         <v>4.9000000000000004</v>
       </c>
       <c r="K12" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" t="s">
         <v>104</v>
+      </c>
+      <c r="D13" t="s">
+        <v>76</v>
+      </c>
+      <c r="E13" t="s">
+        <v>4</v>
+      </c>
+      <c r="F13" t="s">
+        <v>77</v>
+      </c>
+      <c r="G13" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H13" t="s">
+        <v>84</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>5</v>
+      </c>
+      <c r="K13" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB009 Sum of First N Numbers
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC499C6-A34C-4683-B5EF-7E166C102D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C513EDE7-51C4-4A5E-B150-37D1055945E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="109">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -375,6 +375,12 @@
   </si>
   <si>
     <t>Loops, If-Else</t>
+  </si>
+  <si>
+    <t>Sum of First N Numbers</t>
+  </si>
+  <si>
+    <t>Loops, Accumalator</t>
   </si>
 </sst>
 </file>
@@ -1374,6 +1380,36 @@
       <c r="A14">
         <v>13</v>
       </c>
+      <c r="B14" t="s">
+        <v>34</v>
+      </c>
+      <c r="C14" t="s">
+        <v>107</v>
+      </c>
+      <c r="D14" t="s">
+        <v>76</v>
+      </c>
+      <c r="E14" t="s">
+        <v>4</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H14" t="s">
+        <v>84</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>5</v>
+      </c>
+      <c r="K14" t="s">
+        <v>108</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K1" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}"/>

</xml_diff>

<commit_message>
Solved PB010 Fatorial of Number
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C513EDE7-51C4-4A5E-B150-37D1055945E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481DA0BA-C72A-474C-B283-4DDDDDA7A704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="110">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -381,6 +381,9 @@
   </si>
   <si>
     <t>Loops, Accumalator</t>
+  </si>
+  <si>
+    <t>Factorial of number</t>
   </si>
 </sst>
 </file>
@@ -900,7 +903,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1408,6 +1411,41 @@
         <v>5</v>
       </c>
       <c r="K14" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
+        <v>109</v>
+      </c>
+      <c r="D15" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" t="s">
+        <v>4</v>
+      </c>
+      <c r="F15" t="s">
+        <v>77</v>
+      </c>
+      <c r="G15" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H15" t="s">
+        <v>84</v>
+      </c>
+      <c r="I15">
+        <v>1</v>
+      </c>
+      <c r="J15">
+        <v>5</v>
+      </c>
+      <c r="K15" t="s">
         <v>108</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Solved PB011 Prime Number
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{481DA0BA-C72A-474C-B283-4DDDDDA7A704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236A1018-1927-416B-8BBA-C0C4F434AD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="112">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -384,6 +384,12 @@
   </si>
   <si>
     <t>Factorial of number</t>
+  </si>
+  <si>
+    <t>Prime Number</t>
+  </si>
+  <si>
+    <t>Divisibilty</t>
   </si>
 </sst>
 </file>
@@ -903,7 +909,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1447,6 +1453,41 @@
       </c>
       <c r="K15" t="s">
         <v>108</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" t="s">
+        <v>110</v>
+      </c>
+      <c r="D16" t="s">
+        <v>76</v>
+      </c>
+      <c r="E16" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" t="s">
+        <v>77</v>
+      </c>
+      <c r="G16" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H16" t="s">
+        <v>102</v>
+      </c>
+      <c r="I16">
+        <v>1</v>
+      </c>
+      <c r="J16">
+        <v>5</v>
+      </c>
+      <c r="K16" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB012 Fibonacci Series
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{236A1018-1927-416B-8BBA-C0C4F434AD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB4B0C8-536D-4CB8-BE5E-D3203E3AF43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="116">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -390,6 +390,18 @@
   </si>
   <si>
     <t>Divisibilty</t>
+  </si>
+  <si>
+    <t>Number Manipulation</t>
+  </si>
+  <si>
+    <t>Fibonacci Series</t>
+  </si>
+  <si>
+    <t>Easy-Medium</t>
+  </si>
+  <si>
+    <t>Sequence Generation</t>
   </si>
 </sst>
 </file>
@@ -909,7 +921,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1488,6 +1500,41 @@
       </c>
       <c r="K16" t="s">
         <v>111</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>112</v>
+      </c>
+      <c r="C17" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E17" t="s">
+        <v>114</v>
+      </c>
+      <c r="F17" t="s">
+        <v>77</v>
+      </c>
+      <c r="G17" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H17" t="s">
+        <v>102</v>
+      </c>
+      <c r="I17">
+        <v>1</v>
+      </c>
+      <c r="J17">
+        <v>5</v>
+      </c>
+      <c r="K17" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB013 Count Digits
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EB4B0C8-536D-4CB8-BE5E-D3203E3AF43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C69209F-0A55-4A4F-B8F0-8727DB70FF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="118">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -402,6 +402,12 @@
   </si>
   <si>
     <t>Sequence Generation</t>
+  </si>
+  <si>
+    <t>Count Digits</t>
+  </si>
+  <si>
+    <t>Digit Extraction</t>
   </si>
 </sst>
 </file>
@@ -921,7 +927,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1535,6 +1541,41 @@
       </c>
       <c r="K17" t="s">
         <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" t="s">
+        <v>116</v>
+      </c>
+      <c r="D18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E18" t="s">
+        <v>114</v>
+      </c>
+      <c r="F18" t="s">
+        <v>77</v>
+      </c>
+      <c r="G18" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H18" t="s">
+        <v>98</v>
+      </c>
+      <c r="I18">
+        <v>1</v>
+      </c>
+      <c r="J18">
+        <v>5</v>
+      </c>
+      <c r="K18" t="s">
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB014 Sum of Digits
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C69209F-0A55-4A4F-B8F0-8727DB70FF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A854310D-2C7A-4E9F-968C-FF2F92B24AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="120">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -408,6 +408,12 @@
   </si>
   <si>
     <t>Digit Extraction</t>
+  </si>
+  <si>
+    <t>Sum of Digits</t>
+  </si>
+  <si>
+    <t>Digit Extraction, Accumalator</t>
   </si>
 </sst>
 </file>
@@ -927,7 +933,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1576,6 +1582,41 @@
       </c>
       <c r="K18" t="s">
         <v>117</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>112</v>
+      </c>
+      <c r="C19" t="s">
+        <v>118</v>
+      </c>
+      <c r="D19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" t="s">
+        <v>114</v>
+      </c>
+      <c r="F19" t="s">
+        <v>77</v>
+      </c>
+      <c r="G19" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H19" t="s">
+        <v>84</v>
+      </c>
+      <c r="I19">
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <v>5</v>
+      </c>
+      <c r="K19" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB015 Reverse Number
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A854310D-2C7A-4E9F-968C-FF2F92B24AB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A50CFA31-A9A9-4665-8B86-A0C63790C3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4572" yWindow="696" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="-1992" yWindow="852" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="122">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -414,6 +414,12 @@
   </si>
   <si>
     <t>Digit Extraction, Accumalator</t>
+  </si>
+  <si>
+    <t>Reverse Number</t>
+  </si>
+  <si>
+    <t>Digit Extraction, Number Construction</t>
   </si>
 </sst>
 </file>
@@ -933,7 +939,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1617,6 +1623,41 @@
       </c>
       <c r="K19" t="s">
         <v>119</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" t="s">
+        <v>120</v>
+      </c>
+      <c r="D20" t="s">
+        <v>76</v>
+      </c>
+      <c r="E20" t="s">
+        <v>114</v>
+      </c>
+      <c r="F20" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H20" t="s">
+        <v>98</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20">
+        <v>5</v>
+      </c>
+      <c r="K20" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB016 Palindrome Number
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A50CFA31-A9A9-4665-8B86-A0C63790C3D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71847B9A-984F-472A-8A3C-13C71A144690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1992" yWindow="852" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="348" yWindow="936" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="124">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -420,6 +420,12 @@
   </si>
   <si>
     <t>Digit Extraction, Number Construction</t>
+  </si>
+  <si>
+    <t>Palindrome Number</t>
+  </si>
+  <si>
+    <t>Reverse, Compare</t>
   </si>
 </sst>
 </file>
@@ -939,7 +945,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1658,6 +1664,41 @@
       </c>
       <c r="K20" t="s">
         <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" t="s">
+        <v>122</v>
+      </c>
+      <c r="D21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E21" t="s">
+        <v>114</v>
+      </c>
+      <c r="F21" t="s">
+        <v>77</v>
+      </c>
+      <c r="G21" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H21" t="s">
+        <v>84</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>5</v>
+      </c>
+      <c r="K21" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB018 Strong number
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71847B9A-984F-472A-8A3C-13C71A144690}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA024778-7E45-44F4-A4F4-5CF6155C8F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="348" yWindow="936" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="-2688" yWindow="912" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="127">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -426,6 +426,15 @@
   </si>
   <si>
     <t>Reverse, Compare</t>
+  </si>
+  <si>
+    <t>Strong Number</t>
+  </si>
+  <si>
+    <t>6 min</t>
+  </si>
+  <si>
+    <t>Digit Extraction, Nested Loop</t>
   </si>
 </sst>
 </file>
@@ -945,7 +954,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1699,6 +1708,41 @@
       </c>
       <c r="K21" t="s">
         <v>123</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C22" t="s">
+        <v>124</v>
+      </c>
+      <c r="D22" t="s">
+        <v>76</v>
+      </c>
+      <c r="E22" t="s">
+        <v>114</v>
+      </c>
+      <c r="F22" t="s">
+        <v>77</v>
+      </c>
+      <c r="G22" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H22" t="s">
+        <v>125</v>
+      </c>
+      <c r="I22">
+        <v>1</v>
+      </c>
+      <c r="J22">
+        <v>5</v>
+      </c>
+      <c r="K22" t="s">
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB019 Perfect Number
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA024778-7E45-44F4-A4F4-5CF6155C8F77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AD5BCC5-1168-44E9-9377-C9A96ED94DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2688" yWindow="912" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="129">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -435,6 +435,12 @@
   </si>
   <si>
     <t>Digit Extraction, Nested Loop</t>
+  </si>
+  <si>
+    <t>Perfect Number</t>
+  </si>
+  <si>
+    <t>Factor traversal, Accumalator</t>
   </si>
 </sst>
 </file>
@@ -954,7 +960,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1743,6 +1749,41 @@
       </c>
       <c r="K22" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>112</v>
+      </c>
+      <c r="C23" t="s">
+        <v>127</v>
+      </c>
+      <c r="D23" t="s">
+        <v>76</v>
+      </c>
+      <c r="E23" t="s">
+        <v>114</v>
+      </c>
+      <c r="F23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G23" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H23" t="s">
+        <v>102</v>
+      </c>
+      <c r="I23">
+        <v>1</v>
+      </c>
+      <c r="J23">
+        <v>5</v>
+      </c>
+      <c r="K23" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solved PB017 Armstrong Number
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3A5869E-17C6-4E2D-B9F9-22E4CA259C6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF00B3E7-6691-46A5-BB20-50F2D523C15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="135">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -450,6 +450,15 @@
   </si>
   <si>
     <t>LCM</t>
+  </si>
+  <si>
+    <t>Armstrong Number</t>
+  </si>
+  <si>
+    <t>8 min</t>
+  </si>
+  <si>
+    <t>Digit Extraction, Accumalator, Power</t>
   </si>
 </sst>
 </file>
@@ -969,7 +978,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1863,6 +1872,41 @@
       </c>
       <c r="K25" t="s">
         <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>112</v>
+      </c>
+      <c r="C26" t="s">
+        <v>132</v>
+      </c>
+      <c r="D26" t="s">
+        <v>76</v>
+      </c>
+      <c r="E26" t="s">
+        <v>114</v>
+      </c>
+      <c r="F26" t="s">
+        <v>77</v>
+      </c>
+      <c r="G26" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H26" t="s">
+        <v>133</v>
+      </c>
+      <c r="I26">
+        <v>2</v>
+      </c>
+      <c r="J26">
+        <v>4.5</v>
+      </c>
+      <c r="K26" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Complete LeetCode Number Manipulation Easy Problems
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10CD2FF5-1CDA-4646-B0A0-754252D8E321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC64776-992A-4B95-B3FE-B15CB3E936EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="153">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -489,6 +489,30 @@
   </si>
   <si>
     <t>Java String Reverse</t>
+  </si>
+  <si>
+    <t>Leetcode</t>
+  </si>
+  <si>
+    <t>Fibonacci Number</t>
+  </si>
+  <si>
+    <t>Count the digits that divide a number</t>
+  </si>
+  <si>
+    <t>Subtract the product and sum of digits of a number</t>
+  </si>
+  <si>
+    <t>Smallest even multiple</t>
+  </si>
+  <si>
+    <t>Digit extraction, Divisibilty check</t>
+  </si>
+  <si>
+    <t>Digit extraction, Multiple accumalator</t>
+  </si>
+  <si>
+    <t>LCM, Conditional logic</t>
   </si>
 </sst>
 </file>
@@ -1008,7 +1032,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N31"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -2112,6 +2136,216 @@
       </c>
       <c r="K31" t="s">
         <v>141</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>112</v>
+      </c>
+      <c r="C32" t="s">
+        <v>120</v>
+      </c>
+      <c r="D32" t="s">
+        <v>145</v>
+      </c>
+      <c r="E32" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" t="s">
+        <v>77</v>
+      </c>
+      <c r="G32" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H32" t="s">
+        <v>125</v>
+      </c>
+      <c r="I32">
+        <v>1</v>
+      </c>
+      <c r="J32">
+        <v>5</v>
+      </c>
+      <c r="K32" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>112</v>
+      </c>
+      <c r="C33" t="s">
+        <v>122</v>
+      </c>
+      <c r="D33" t="s">
+        <v>145</v>
+      </c>
+      <c r="E33" t="s">
+        <v>4</v>
+      </c>
+      <c r="F33" t="s">
+        <v>77</v>
+      </c>
+      <c r="G33" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H33" t="s">
+        <v>102</v>
+      </c>
+      <c r="I33">
+        <v>1</v>
+      </c>
+      <c r="J33">
+        <v>5</v>
+      </c>
+      <c r="K33" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" t="s">
+        <v>146</v>
+      </c>
+      <c r="D34" t="s">
+        <v>145</v>
+      </c>
+      <c r="E34" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" t="s">
+        <v>77</v>
+      </c>
+      <c r="G34" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H34" t="s">
+        <v>98</v>
+      </c>
+      <c r="I34">
+        <v>1</v>
+      </c>
+      <c r="J34">
+        <v>5</v>
+      </c>
+      <c r="K34" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>112</v>
+      </c>
+      <c r="C35" t="s">
+        <v>147</v>
+      </c>
+      <c r="D35" t="s">
+        <v>145</v>
+      </c>
+      <c r="E35" t="s">
+        <v>4</v>
+      </c>
+      <c r="F35" t="s">
+        <v>77</v>
+      </c>
+      <c r="G35" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H35" t="s">
+        <v>84</v>
+      </c>
+      <c r="I35">
+        <v>1</v>
+      </c>
+      <c r="J35">
+        <v>5</v>
+      </c>
+      <c r="K35" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>112</v>
+      </c>
+      <c r="C36" t="s">
+        <v>148</v>
+      </c>
+      <c r="D36" t="s">
+        <v>145</v>
+      </c>
+      <c r="E36" t="s">
+        <v>4</v>
+      </c>
+      <c r="F36" t="s">
+        <v>77</v>
+      </c>
+      <c r="G36" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H36" t="s">
+        <v>84</v>
+      </c>
+      <c r="I36">
+        <v>1</v>
+      </c>
+      <c r="J36">
+        <v>5</v>
+      </c>
+      <c r="K36" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>112</v>
+      </c>
+      <c r="C37" t="s">
+        <v>149</v>
+      </c>
+      <c r="D37" t="s">
+        <v>145</v>
+      </c>
+      <c r="E37" t="s">
+        <v>4</v>
+      </c>
+      <c r="F37" t="s">
+        <v>77</v>
+      </c>
+      <c r="G37" s="2">
+        <v>46190</v>
+      </c>
+      <c r="H37" t="s">
+        <v>102</v>
+      </c>
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37">
+        <v>5</v>
+      </c>
+      <c r="K37" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB022  Square Pattern
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC64776-992A-4B95-B3FE-B15CB3E936EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F5FF29-C387-4AA9-9A09-B47FCA1389D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="174">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -513,6 +513,69 @@
   </si>
   <si>
     <t>LCM, Conditional logic</t>
+  </si>
+  <si>
+    <t>Pattern Printing</t>
+  </si>
+  <si>
+    <t>Square Pattern</t>
+  </si>
+  <si>
+    <t>Hollow sqaure</t>
+  </si>
+  <si>
+    <t>Right triangle</t>
+  </si>
+  <si>
+    <t>inverted triangle</t>
+  </si>
+  <si>
+    <t>number triangle</t>
+  </si>
+  <si>
+    <t>Floyd's triangle</t>
+  </si>
+  <si>
+    <t>pyramid</t>
+  </si>
+  <si>
+    <t>inverted pyramid</t>
+  </si>
+  <si>
+    <t>Diamond</t>
+  </si>
+  <si>
+    <t>butterfly Pattern</t>
+  </si>
+  <si>
+    <t>Nested Loop</t>
+  </si>
+  <si>
+    <t>Boundary Conditions</t>
+  </si>
+  <si>
+    <t>Row-Column Logic</t>
+  </si>
+  <si>
+    <t>Reverse Loop</t>
+  </si>
+  <si>
+    <t>Nested Loop, Numbers</t>
+  </si>
+  <si>
+    <t>Running Counter</t>
+  </si>
+  <si>
+    <t>Spaces, stars</t>
+  </si>
+  <si>
+    <t>Reverse Pattern</t>
+  </si>
+  <si>
+    <t>Upper, Lower Half</t>
+  </si>
+  <si>
+    <t>Symmetry</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1095,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -2346,6 +2409,194 @@
       </c>
       <c r="K37" t="s">
         <v>152</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>153</v>
+      </c>
+      <c r="C38" t="s">
+        <v>154</v>
+      </c>
+      <c r="D38" t="s">
+        <v>76</v>
+      </c>
+      <c r="E38" t="s">
+        <v>114</v>
+      </c>
+      <c r="F38" t="s">
+        <v>77</v>
+      </c>
+      <c r="G38" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H38" t="s">
+        <v>98</v>
+      </c>
+      <c r="I38">
+        <v>1</v>
+      </c>
+      <c r="J38">
+        <v>5</v>
+      </c>
+      <c r="K38" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>153</v>
+      </c>
+      <c r="C39" t="s">
+        <v>155</v>
+      </c>
+      <c r="D39" t="s">
+        <v>76</v>
+      </c>
+      <c r="K39" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>153</v>
+      </c>
+      <c r="C40" t="s">
+        <v>156</v>
+      </c>
+      <c r="D40" t="s">
+        <v>76</v>
+      </c>
+      <c r="K40" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>153</v>
+      </c>
+      <c r="C41" t="s">
+        <v>157</v>
+      </c>
+      <c r="D41" t="s">
+        <v>76</v>
+      </c>
+      <c r="K41" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>153</v>
+      </c>
+      <c r="C42" t="s">
+        <v>158</v>
+      </c>
+      <c r="D42" t="s">
+        <v>76</v>
+      </c>
+      <c r="K42" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>153</v>
+      </c>
+      <c r="C43" t="s">
+        <v>159</v>
+      </c>
+      <c r="D43" t="s">
+        <v>76</v>
+      </c>
+      <c r="K43" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>153</v>
+      </c>
+      <c r="C44" t="s">
+        <v>160</v>
+      </c>
+      <c r="D44" t="s">
+        <v>76</v>
+      </c>
+      <c r="K44" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>153</v>
+      </c>
+      <c r="C45" t="s">
+        <v>161</v>
+      </c>
+      <c r="D45" t="s">
+        <v>76</v>
+      </c>
+      <c r="K45" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>153</v>
+      </c>
+      <c r="C46" t="s">
+        <v>162</v>
+      </c>
+      <c r="D46" t="s">
+        <v>76</v>
+      </c>
+      <c r="K46" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>153</v>
+      </c>
+      <c r="C47" t="s">
+        <v>163</v>
+      </c>
+      <c r="D47" t="s">
+        <v>76</v>
+      </c>
+      <c r="K47" t="s">
+        <v>173</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB023  Hollow Square Pattern
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97F5FF29-C387-4AA9-9A09-B47FCA1389D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA5A774-9D8A-4321-903E-23FEEAE343B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="174">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -2459,6 +2459,24 @@
       <c r="D39" t="s">
         <v>76</v>
       </c>
+      <c r="E39" t="s">
+        <v>5</v>
+      </c>
+      <c r="F39" t="s">
+        <v>77</v>
+      </c>
+      <c r="G39" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H39" t="s">
+        <v>133</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39">
+        <v>4.8</v>
+      </c>
       <c r="K39" t="s">
         <v>165</v>
       </c>

</xml_diff>

<commit_message>
Solve PB024  Right Triangle Pattern
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BA5A774-9D8A-4321-903E-23FEEAE343B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5826341D-76AE-49A5-BE12-DBACF123F853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="174">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -2494,6 +2494,24 @@
       <c r="D40" t="s">
         <v>76</v>
       </c>
+      <c r="E40" t="s">
+        <v>114</v>
+      </c>
+      <c r="F40" t="s">
+        <v>77</v>
+      </c>
+      <c r="G40" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H40" t="s">
+        <v>102</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="J40">
+        <v>5</v>
+      </c>
       <c r="K40" t="s">
         <v>166</v>
       </c>

</xml_diff>

<commit_message>
Solve PB025  Inverted Right Triangle
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5826341D-76AE-49A5-BE12-DBACF123F853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E12A612-9421-4233-8ACA-6020958B8C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="174">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -2529,6 +2529,24 @@
       <c r="D41" t="s">
         <v>76</v>
       </c>
+      <c r="E41" t="s">
+        <v>114</v>
+      </c>
+      <c r="F41" t="s">
+        <v>77</v>
+      </c>
+      <c r="G41" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H41" t="s">
+        <v>98</v>
+      </c>
+      <c r="I41">
+        <v>1</v>
+      </c>
+      <c r="J41">
+        <v>5</v>
+      </c>
       <c r="K41" t="s">
         <v>167</v>
       </c>

</xml_diff>

<commit_message>
Solve PB026  Number Triangle Pattern
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E12A612-9421-4233-8ACA-6020958B8C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5DEE07-FDDC-49B4-BF10-0A777EAFB73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="405" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="174">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -2564,6 +2564,24 @@
       <c r="D42" t="s">
         <v>76</v>
       </c>
+      <c r="E42" t="s">
+        <v>114</v>
+      </c>
+      <c r="F42" t="s">
+        <v>77</v>
+      </c>
+      <c r="G42" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H42" t="s">
+        <v>102</v>
+      </c>
+      <c r="I42">
+        <v>1</v>
+      </c>
+      <c r="J42">
+        <v>5</v>
+      </c>
       <c r="K42" t="s">
         <v>168</v>
       </c>

</xml_diff>

<commit_message>
Solve PB027  Floyd's Triangle
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D5DEE07-FDDC-49B4-BF10-0A777EAFB73F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{298B6760-B1E3-4B0B-810D-BA8276C1763F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="174">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -2599,6 +2599,24 @@
       <c r="D43" t="s">
         <v>76</v>
       </c>
+      <c r="E43" t="s">
+        <v>114</v>
+      </c>
+      <c r="F43" t="s">
+        <v>77</v>
+      </c>
+      <c r="G43" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H43" t="s">
+        <v>98</v>
+      </c>
+      <c r="I43">
+        <v>1</v>
+      </c>
+      <c r="J43">
+        <v>5</v>
+      </c>
       <c r="K43" t="s">
         <v>169</v>
       </c>

</xml_diff>

<commit_message>
Solve PB028  Pyramid Pattern
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{298B6760-B1E3-4B0B-810D-BA8276C1763F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF18E49-2C3B-427D-B9BA-A4A9DBF31BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="176">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -576,6 +576,12 @@
   </si>
   <si>
     <t>Symmetry</t>
+  </si>
+  <si>
+    <t>10 min</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -2634,6 +2640,24 @@
       <c r="D44" t="s">
         <v>76</v>
       </c>
+      <c r="E44" t="s">
+        <v>5</v>
+      </c>
+      <c r="F44" t="s">
+        <v>77</v>
+      </c>
+      <c r="G44" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H44" t="s">
+        <v>174</v>
+      </c>
+      <c r="I44">
+        <v>3</v>
+      </c>
+      <c r="J44">
+        <v>4.3</v>
+      </c>
       <c r="K44" t="s">
         <v>170</v>
       </c>
@@ -2650,6 +2674,9 @@
       </c>
       <c r="D45" t="s">
         <v>76</v>
+      </c>
+      <c r="G45" t="s">
+        <v>175</v>
       </c>
       <c r="K45" t="s">
         <v>171</v>

</xml_diff>

<commit_message>
Solve PB029 Inverted Pyramid
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF18E49-2C3B-427D-B9BA-A4A9DBF31BFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC0546B2-F9A3-4EBB-9637-853FBDF3883A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12" yWindow="648" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="6540" yWindow="792" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="176">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -581,7 +581,7 @@
     <t>10 min</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t>15 min</t>
   </si>
 </sst>
 </file>
@@ -2675,8 +2675,23 @@
       <c r="D45" t="s">
         <v>76</v>
       </c>
-      <c r="G45" t="s">
+      <c r="E45" t="s">
+        <v>5</v>
+      </c>
+      <c r="F45" t="s">
+        <v>77</v>
+      </c>
+      <c r="G45" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H45" t="s">
         <v>175</v>
+      </c>
+      <c r="I45">
+        <v>5</v>
+      </c>
+      <c r="J45">
+        <v>4</v>
       </c>
       <c r="K45" t="s">
         <v>171</v>

</xml_diff>

<commit_message>
Solve PB030 Diamond Pattern
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC0546B2-F9A3-4EBB-9637-853FBDF3883A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BEC781-449A-4333-9CE8-1B133ED936FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6540" yWindow="792" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="178">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -582,6 +582,12 @@
   </si>
   <si>
     <t>15 min</t>
+  </si>
+  <si>
+    <t>Medium-Hard</t>
+  </si>
+  <si>
+    <t>20 min</t>
   </si>
 </sst>
 </file>
@@ -2710,6 +2716,24 @@
       <c r="D46" t="s">
         <v>76</v>
       </c>
+      <c r="E46" t="s">
+        <v>176</v>
+      </c>
+      <c r="F46" t="s">
+        <v>77</v>
+      </c>
+      <c r="G46" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H46" t="s">
+        <v>177</v>
+      </c>
+      <c r="I46">
+        <v>2</v>
+      </c>
+      <c r="J46">
+        <v>4.5</v>
+      </c>
       <c r="K46" t="s">
         <v>172</v>
       </c>

</xml_diff>

<commit_message>
Complete PB031  Butterfly Pattern
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50BEC781-449A-4333-9CE8-1B133ED936FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888FFB37-AB6A-4FB5-A523-07EDA9410796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6540" yWindow="792" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="179">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -588,6 +588,9 @@
   </si>
   <si>
     <t>20 min</t>
+  </si>
+  <si>
+    <t>25 min</t>
   </si>
 </sst>
 </file>
@@ -2751,6 +2754,24 @@
       <c r="D47" t="s">
         <v>76</v>
       </c>
+      <c r="E47" t="s">
+        <v>6</v>
+      </c>
+      <c r="F47" t="s">
+        <v>77</v>
+      </c>
+      <c r="G47" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H47" t="s">
+        <v>178</v>
+      </c>
+      <c r="I47">
+        <v>5</v>
+      </c>
+      <c r="J47">
+        <v>3.7</v>
+      </c>
       <c r="K47" t="s">
         <v>173</v>
       </c>

</xml_diff>

<commit_message>
Solved Problems on Leetcode and HackerRank
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{888FFB37-AB6A-4FB5-A523-07EDA9410796}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76F14B2-8218-4AE1-8B09-1FAE65CAD9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6540" yWindow="792" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="208">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -591,6 +591,93 @@
   </si>
   <si>
     <t>25 min</t>
+  </si>
+  <si>
+    <t>Java Output Formatting</t>
+  </si>
+  <si>
+    <t>Java Static Initializer block</t>
+  </si>
+  <si>
+    <t>Java Date and Time</t>
+  </si>
+  <si>
+    <t>Java Currency Formatter</t>
+  </si>
+  <si>
+    <t>Java String Introduction</t>
+  </si>
+  <si>
+    <t>Java Substring</t>
+  </si>
+  <si>
+    <t>Java Substring comparison</t>
+  </si>
+  <si>
+    <t>Loops, Formatting</t>
+  </si>
+  <si>
+    <t>Basic Conditions</t>
+  </si>
+  <si>
+    <t>Basic Logic</t>
+  </si>
+  <si>
+    <t>Formatting</t>
+  </si>
+  <si>
+    <t>String Operations</t>
+  </si>
+  <si>
+    <t>String Basics</t>
+  </si>
+  <si>
+    <t>Loops, String traversal</t>
+  </si>
+  <si>
+    <t>Number of Steps to reduce number to zero</t>
+  </si>
+  <si>
+    <t>Add two integers</t>
+  </si>
+  <si>
+    <t>Number after double reversal</t>
+  </si>
+  <si>
+    <t>Convert the temperature</t>
+  </si>
+  <si>
+    <t>Add digits</t>
+  </si>
+  <si>
+    <t>sum multiples</t>
+  </si>
+  <si>
+    <t>self dividing numbers</t>
+  </si>
+  <si>
+    <t>power of two</t>
+  </si>
+  <si>
+    <t>power of three</t>
+  </si>
+  <si>
+    <t>power of four</t>
+  </si>
+  <si>
+    <t>Arithmetic</t>
+  </si>
+  <si>
+    <t>Reverse number</t>
+  </si>
+  <si>
+    <t>formulae based</t>
+  </si>
+  <si>
+    <t>Digit traversal</t>
+  </si>
+  <si>
+    <t>Repeated Division</t>
   </si>
 </sst>
 </file>
@@ -1110,7 +1197,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -2774,6 +2861,636 @@
       </c>
       <c r="K47" t="s">
         <v>173</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>34</v>
+      </c>
+      <c r="C48" t="s">
+        <v>179</v>
+      </c>
+      <c r="D48" t="s">
+        <v>81</v>
+      </c>
+      <c r="E48" t="s">
+        <v>4</v>
+      </c>
+      <c r="F48" t="s">
+        <v>77</v>
+      </c>
+      <c r="G48" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H48" t="s">
+        <v>84</v>
+      </c>
+      <c r="I48">
+        <v>1</v>
+      </c>
+      <c r="J48">
+        <v>5</v>
+      </c>
+      <c r="K48" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>34</v>
+      </c>
+      <c r="C49" t="s">
+        <v>180</v>
+      </c>
+      <c r="D49" t="s">
+        <v>81</v>
+      </c>
+      <c r="E49" t="s">
+        <v>4</v>
+      </c>
+      <c r="F49" t="s">
+        <v>77</v>
+      </c>
+      <c r="G49" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H49" t="s">
+        <v>97</v>
+      </c>
+      <c r="I49">
+        <v>1</v>
+      </c>
+      <c r="J49">
+        <v>5</v>
+      </c>
+      <c r="K49" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>34</v>
+      </c>
+      <c r="C50" t="s">
+        <v>181</v>
+      </c>
+      <c r="D50" t="s">
+        <v>81</v>
+      </c>
+      <c r="E50" t="s">
+        <v>4</v>
+      </c>
+      <c r="F50" t="s">
+        <v>77</v>
+      </c>
+      <c r="G50" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H50" t="s">
+        <v>84</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+      <c r="J50">
+        <v>5</v>
+      </c>
+      <c r="K50" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>34</v>
+      </c>
+      <c r="C51" t="s">
+        <v>182</v>
+      </c>
+      <c r="D51" t="s">
+        <v>81</v>
+      </c>
+      <c r="E51" t="s">
+        <v>4</v>
+      </c>
+      <c r="F51" t="s">
+        <v>77</v>
+      </c>
+      <c r="G51" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H51" t="s">
+        <v>102</v>
+      </c>
+      <c r="I51">
+        <v>1</v>
+      </c>
+      <c r="J51">
+        <v>5</v>
+      </c>
+      <c r="K51" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>34</v>
+      </c>
+      <c r="C52" t="s">
+        <v>183</v>
+      </c>
+      <c r="D52" t="s">
+        <v>81</v>
+      </c>
+      <c r="E52" t="s">
+        <v>4</v>
+      </c>
+      <c r="F52" t="s">
+        <v>77</v>
+      </c>
+      <c r="G52" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H52" t="s">
+        <v>97</v>
+      </c>
+      <c r="I52">
+        <v>1</v>
+      </c>
+      <c r="J52">
+        <v>5</v>
+      </c>
+      <c r="K52" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>34</v>
+      </c>
+      <c r="C53" t="s">
+        <v>184</v>
+      </c>
+      <c r="D53" t="s">
+        <v>81</v>
+      </c>
+      <c r="E53" t="s">
+        <v>4</v>
+      </c>
+      <c r="F53" t="s">
+        <v>77</v>
+      </c>
+      <c r="G53" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H53" t="s">
+        <v>97</v>
+      </c>
+      <c r="I53">
+        <v>1</v>
+      </c>
+      <c r="J53">
+        <v>5</v>
+      </c>
+      <c r="K53" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>34</v>
+      </c>
+      <c r="C54" t="s">
+        <v>185</v>
+      </c>
+      <c r="D54" t="s">
+        <v>81</v>
+      </c>
+      <c r="E54" t="s">
+        <v>4</v>
+      </c>
+      <c r="F54" t="s">
+        <v>77</v>
+      </c>
+      <c r="G54" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H54" t="s">
+        <v>102</v>
+      </c>
+      <c r="I54">
+        <v>1</v>
+      </c>
+      <c r="J54">
+        <v>5</v>
+      </c>
+      <c r="K54" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>112</v>
+      </c>
+      <c r="C55" t="s">
+        <v>193</v>
+      </c>
+      <c r="D55" t="s">
+        <v>145</v>
+      </c>
+      <c r="E55" t="s">
+        <v>4</v>
+      </c>
+      <c r="F55" t="s">
+        <v>77</v>
+      </c>
+      <c r="G55" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H55" t="s">
+        <v>84</v>
+      </c>
+      <c r="I55">
+        <v>1</v>
+      </c>
+      <c r="J55">
+        <v>5</v>
+      </c>
+      <c r="K55" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>112</v>
+      </c>
+      <c r="C56" t="s">
+        <v>194</v>
+      </c>
+      <c r="D56" t="s">
+        <v>145</v>
+      </c>
+      <c r="E56" t="s">
+        <v>4</v>
+      </c>
+      <c r="F56" t="s">
+        <v>77</v>
+      </c>
+      <c r="G56" s="2">
+        <v>46191</v>
+      </c>
+      <c r="H56" t="s">
+        <v>82</v>
+      </c>
+      <c r="I56">
+        <v>1</v>
+      </c>
+      <c r="J56">
+        <v>5</v>
+      </c>
+      <c r="K56" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>112</v>
+      </c>
+      <c r="C57" t="s">
+        <v>195</v>
+      </c>
+      <c r="D57" t="s">
+        <v>145</v>
+      </c>
+      <c r="E57" t="s">
+        <v>4</v>
+      </c>
+      <c r="F57" t="s">
+        <v>77</v>
+      </c>
+      <c r="G57" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H57" t="s">
+        <v>98</v>
+      </c>
+      <c r="I57">
+        <v>1</v>
+      </c>
+      <c r="J57">
+        <v>5</v>
+      </c>
+      <c r="K57" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>112</v>
+      </c>
+      <c r="C58" t="s">
+        <v>196</v>
+      </c>
+      <c r="D58" t="s">
+        <v>145</v>
+      </c>
+      <c r="E58" t="s">
+        <v>4</v>
+      </c>
+      <c r="F58" t="s">
+        <v>77</v>
+      </c>
+      <c r="G58" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H58" t="s">
+        <v>97</v>
+      </c>
+      <c r="I58">
+        <v>1</v>
+      </c>
+      <c r="J58">
+        <v>5</v>
+      </c>
+      <c r="K58" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>112</v>
+      </c>
+      <c r="C59" t="s">
+        <v>197</v>
+      </c>
+      <c r="D59" t="s">
+        <v>145</v>
+      </c>
+      <c r="E59" t="s">
+        <v>4</v>
+      </c>
+      <c r="F59" t="s">
+        <v>77</v>
+      </c>
+      <c r="G59" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H59" t="s">
+        <v>98</v>
+      </c>
+      <c r="I59">
+        <v>1</v>
+      </c>
+      <c r="J59">
+        <v>5</v>
+      </c>
+      <c r="K59" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>112</v>
+      </c>
+      <c r="C60" t="s">
+        <v>198</v>
+      </c>
+      <c r="D60" t="s">
+        <v>145</v>
+      </c>
+      <c r="E60" t="s">
+        <v>4</v>
+      </c>
+      <c r="F60" t="s">
+        <v>77</v>
+      </c>
+      <c r="G60" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H60" t="s">
+        <v>98</v>
+      </c>
+      <c r="I60">
+        <v>1</v>
+      </c>
+      <c r="J60">
+        <v>5</v>
+      </c>
+      <c r="K60" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>112</v>
+      </c>
+      <c r="C61" t="s">
+        <v>199</v>
+      </c>
+      <c r="D61" t="s">
+        <v>145</v>
+      </c>
+      <c r="E61" t="s">
+        <v>4</v>
+      </c>
+      <c r="F61" t="s">
+        <v>77</v>
+      </c>
+      <c r="G61" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H61" t="s">
+        <v>102</v>
+      </c>
+      <c r="I61">
+        <v>1</v>
+      </c>
+      <c r="J61">
+        <v>5</v>
+      </c>
+      <c r="K61" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>112</v>
+      </c>
+      <c r="C62" t="s">
+        <v>127</v>
+      </c>
+      <c r="D62" t="s">
+        <v>145</v>
+      </c>
+      <c r="E62" t="s">
+        <v>4</v>
+      </c>
+      <c r="F62" t="s">
+        <v>77</v>
+      </c>
+      <c r="G62" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H62" t="s">
+        <v>98</v>
+      </c>
+      <c r="I62">
+        <v>1</v>
+      </c>
+      <c r="J62">
+        <v>5</v>
+      </c>
+      <c r="K62" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" t="s">
+        <v>200</v>
+      </c>
+      <c r="D63" t="s">
+        <v>145</v>
+      </c>
+      <c r="E63" t="s">
+        <v>4</v>
+      </c>
+      <c r="F63" t="s">
+        <v>77</v>
+      </c>
+      <c r="G63" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H63" t="s">
+        <v>84</v>
+      </c>
+      <c r="I63">
+        <v>1</v>
+      </c>
+      <c r="J63">
+        <v>5</v>
+      </c>
+      <c r="K63" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>112</v>
+      </c>
+      <c r="C64" t="s">
+        <v>201</v>
+      </c>
+      <c r="D64" t="s">
+        <v>145</v>
+      </c>
+      <c r="E64" t="s">
+        <v>4</v>
+      </c>
+      <c r="F64" t="s">
+        <v>77</v>
+      </c>
+      <c r="G64" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H64" t="s">
+        <v>84</v>
+      </c>
+      <c r="I64">
+        <v>1</v>
+      </c>
+      <c r="J64">
+        <v>5</v>
+      </c>
+      <c r="K64" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>112</v>
+      </c>
+      <c r="C65" t="s">
+        <v>202</v>
+      </c>
+      <c r="D65" t="s">
+        <v>145</v>
+      </c>
+      <c r="E65" t="s">
+        <v>4</v>
+      </c>
+      <c r="F65" t="s">
+        <v>77</v>
+      </c>
+      <c r="G65" s="2">
+        <v>46192</v>
+      </c>
+      <c r="H65" t="s">
+        <v>84</v>
+      </c>
+      <c r="I65">
+        <v>1</v>
+      </c>
+      <c r="J65">
+        <v>5</v>
+      </c>
+      <c r="K65" t="s">
+        <v>207</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB032 - Read and Print Array
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A76F14B2-8218-4AE1-8B09-1FAE65CAD9B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E17FC0A-4ECA-42CA-8717-9E861C57E7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="6660" yWindow="4200" windowWidth="17280" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="210">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -678,6 +678,12 @@
   </si>
   <si>
     <t>Repeated Division</t>
+  </si>
+  <si>
+    <t>Read and Print Array</t>
+  </si>
+  <si>
+    <t>Array Traversal</t>
   </si>
 </sst>
 </file>
@@ -1197,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3491,6 +3497,41 @@
       </c>
       <c r="K65" t="s">
         <v>207</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>36</v>
+      </c>
+      <c r="C66" t="s">
+        <v>208</v>
+      </c>
+      <c r="D66" t="s">
+        <v>76</v>
+      </c>
+      <c r="E66" t="s">
+        <v>4</v>
+      </c>
+      <c r="F66" t="s">
+        <v>77</v>
+      </c>
+      <c r="G66" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H66" t="s">
+        <v>98</v>
+      </c>
+      <c r="I66">
+        <v>1</v>
+      </c>
+      <c r="J66">
+        <v>5</v>
+      </c>
+      <c r="K66" t="s">
+        <v>209</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB033 - Sum of Array Elements
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E17FC0A-4ECA-42CA-8717-9E861C57E7DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C36847B-5FA8-4E33-B85D-D70BB5BAD589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6660" yWindow="4200" windowWidth="17280" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="212">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -684,6 +684,12 @@
   </si>
   <si>
     <t>Array Traversal</t>
+  </si>
+  <si>
+    <t>Sum of Element of Array</t>
+  </si>
+  <si>
+    <t>Traversal, Accumalator</t>
   </si>
 </sst>
 </file>
@@ -1203,7 +1209,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N67"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3532,6 +3538,41 @@
       </c>
       <c r="K66" t="s">
         <v>209</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>36</v>
+      </c>
+      <c r="C67" t="s">
+        <v>210</v>
+      </c>
+      <c r="D67" t="s">
+        <v>76</v>
+      </c>
+      <c r="E67" t="s">
+        <v>4</v>
+      </c>
+      <c r="F67" t="s">
+        <v>77</v>
+      </c>
+      <c r="G67" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H67" t="s">
+        <v>102</v>
+      </c>
+      <c r="I67">
+        <v>1</v>
+      </c>
+      <c r="J67">
+        <v>5</v>
+      </c>
+      <c r="K67" t="s">
+        <v>211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB034 - Largest Element
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C36847B-5FA8-4E33-B85D-D70BB5BAD589}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77F2CA2-0E19-49CB-B08E-998A96E86F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6660" yWindow="4200" windowWidth="17280" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="214">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -690,6 +690,12 @@
   </si>
   <si>
     <t>Traversal, Accumalator</t>
+  </si>
+  <si>
+    <t>Largest Element</t>
+  </si>
+  <si>
+    <t>Traversal, Maximum Tracking</t>
   </si>
 </sst>
 </file>
@@ -1209,7 +1215,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N67"/>
+  <dimension ref="A1:N68"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3573,6 +3579,41 @@
       </c>
       <c r="K67" t="s">
         <v>211</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>36</v>
+      </c>
+      <c r="C68" t="s">
+        <v>212</v>
+      </c>
+      <c r="D68" t="s">
+        <v>76</v>
+      </c>
+      <c r="E68" t="s">
+        <v>4</v>
+      </c>
+      <c r="F68" t="s">
+        <v>77</v>
+      </c>
+      <c r="G68" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H68" t="s">
+        <v>133</v>
+      </c>
+      <c r="I68">
+        <v>1</v>
+      </c>
+      <c r="J68">
+        <v>5</v>
+      </c>
+      <c r="K68" t="s">
+        <v>213</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB035 - Smallest Element
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77F2CA2-0E19-49CB-B08E-998A96E86F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A748DE05-6356-43F1-B9C6-80FA8EBE9EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6660" yWindow="4200" windowWidth="17280" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="217">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -696,6 +696,15 @@
   </si>
   <si>
     <t>Traversal, Maximum Tracking</t>
+  </si>
+  <si>
+    <t>Smallest Element</t>
+  </si>
+  <si>
+    <t>7 min</t>
+  </si>
+  <si>
+    <t>Traversal, Minimum Tracking</t>
   </si>
 </sst>
 </file>
@@ -1215,7 +1224,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3614,6 +3623,41 @@
       </c>
       <c r="K68" t="s">
         <v>213</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>36</v>
+      </c>
+      <c r="C69" t="s">
+        <v>214</v>
+      </c>
+      <c r="D69" t="s">
+        <v>76</v>
+      </c>
+      <c r="E69" t="s">
+        <v>4</v>
+      </c>
+      <c r="F69" t="s">
+        <v>77</v>
+      </c>
+      <c r="G69" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H69" t="s">
+        <v>215</v>
+      </c>
+      <c r="I69">
+        <v>1</v>
+      </c>
+      <c r="J69">
+        <v>5</v>
+      </c>
+      <c r="K69" t="s">
+        <v>216</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB036  Second Largest Element
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A748DE05-6356-43F1-B9C6-80FA8EBE9EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D34CB4D-1BC0-4FD1-9061-5D1864BB8969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="4200" windowWidth="17280" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="4644" yWindow="4200" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="577" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="219">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -705,6 +705,12 @@
   </si>
   <si>
     <t>Traversal, Minimum Tracking</t>
+  </si>
+  <si>
+    <t>Second Largest Element in array</t>
+  </si>
+  <si>
+    <t>Traversal, Double Variable tracking</t>
   </si>
 </sst>
 </file>
@@ -1224,7 +1230,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N69"/>
+  <dimension ref="A1:N70"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3658,6 +3664,41 @@
       </c>
       <c r="K69" t="s">
         <v>216</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>36</v>
+      </c>
+      <c r="C70" t="s">
+        <v>217</v>
+      </c>
+      <c r="D70" t="s">
+        <v>76</v>
+      </c>
+      <c r="E70" t="s">
+        <v>114</v>
+      </c>
+      <c r="F70" t="s">
+        <v>77</v>
+      </c>
+      <c r="G70" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H70" t="s">
+        <v>174</v>
+      </c>
+      <c r="I70">
+        <v>1</v>
+      </c>
+      <c r="J70">
+        <v>5</v>
+      </c>
+      <c r="K70" t="s">
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB037 - Reverse Array
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D34CB4D-1BC0-4FD1-9061-5D1864BB8969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE37674-C202-45F4-B1CF-061F58552670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4644" yWindow="4200" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="221">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -711,6 +711,12 @@
   </si>
   <si>
     <t>Traversal, Double Variable tracking</t>
+  </si>
+  <si>
+    <t>Reverse Array</t>
+  </si>
+  <si>
+    <t>Two Pointer technique</t>
   </si>
 </sst>
 </file>
@@ -1230,7 +1236,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3699,6 +3705,41 @@
       </c>
       <c r="K70" t="s">
         <v>218</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>36</v>
+      </c>
+      <c r="C71" t="s">
+        <v>219</v>
+      </c>
+      <c r="D71" t="s">
+        <v>76</v>
+      </c>
+      <c r="E71" t="s">
+        <v>114</v>
+      </c>
+      <c r="F71" t="s">
+        <v>77</v>
+      </c>
+      <c r="G71" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H71" t="s">
+        <v>133</v>
+      </c>
+      <c r="I71">
+        <v>1</v>
+      </c>
+      <c r="J71">
+        <v>5</v>
+      </c>
+      <c r="K71" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB038 - Linear Search
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE37674-C202-45F4-B1CF-061F58552670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40567921-11A7-408D-923E-7B8D0A8E7DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4644" yWindow="4200" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="221">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="223">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -717,6 +717,12 @@
   </si>
   <si>
     <t>Two Pointer technique</t>
+  </si>
+  <si>
+    <t>Linear search</t>
+  </si>
+  <si>
+    <t>Linear Search + Flag variable</t>
   </si>
 </sst>
 </file>
@@ -1236,7 +1242,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3740,6 +3746,41 @@
       </c>
       <c r="K71" t="s">
         <v>220</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>36</v>
+      </c>
+      <c r="C72" t="s">
+        <v>221</v>
+      </c>
+      <c r="D72" t="s">
+        <v>76</v>
+      </c>
+      <c r="E72" t="s">
+        <v>114</v>
+      </c>
+      <c r="F72" t="s">
+        <v>77</v>
+      </c>
+      <c r="G72" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H72" t="s">
+        <v>125</v>
+      </c>
+      <c r="I72">
+        <v>1</v>
+      </c>
+      <c r="J72">
+        <v>5</v>
+      </c>
+      <c r="K72" t="s">
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB039 - Count Even and Odd Elements
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40567921-11A7-408D-923E-7B8D0A8E7DE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63B71F49-2EBA-4EB5-85F9-26C5126A1279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4644" yWindow="4200" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="0" yWindow="3360" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="598" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="225">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -723,6 +723,12 @@
   </si>
   <si>
     <t>Linear Search + Flag variable</t>
+  </si>
+  <si>
+    <t>Count Even &amp; Odd Digits</t>
+  </si>
+  <si>
+    <t>Traversal, Multiple Accumalator</t>
   </si>
 </sst>
 </file>
@@ -1242,7 +1248,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N72"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3781,6 +3787,41 @@
       </c>
       <c r="K72" t="s">
         <v>222</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>36</v>
+      </c>
+      <c r="C73" t="s">
+        <v>223</v>
+      </c>
+      <c r="D73" t="s">
+        <v>76</v>
+      </c>
+      <c r="E73" t="s">
+        <v>114</v>
+      </c>
+      <c r="F73" t="s">
+        <v>77</v>
+      </c>
+      <c r="G73" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H73" t="s">
+        <v>102</v>
+      </c>
+      <c r="I73">
+        <v>1</v>
+      </c>
+      <c r="J73">
+        <v>5</v>
+      </c>
+      <c r="K73" t="s">
+        <v>224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB040 - Check if Array is Sorted
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63B71F49-2EBA-4EB5-85F9-26C5126A1279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0F40E9-CD5B-40D8-9ED4-F95529500272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="3360" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="605" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="227">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -729,6 +729,12 @@
   </si>
   <si>
     <t>Traversal, Multiple Accumalator</t>
+  </si>
+  <si>
+    <t>Check if array is sorted or not</t>
+  </si>
+  <si>
+    <t>Adajcent Element comparison</t>
   </si>
 </sst>
 </file>
@@ -1248,7 +1254,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N74"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3822,6 +3828,41 @@
       </c>
       <c r="K73" t="s">
         <v>224</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>36</v>
+      </c>
+      <c r="C74" t="s">
+        <v>225</v>
+      </c>
+      <c r="D74" t="s">
+        <v>76</v>
+      </c>
+      <c r="E74" t="s">
+        <v>114</v>
+      </c>
+      <c r="F74" t="s">
+        <v>77</v>
+      </c>
+      <c r="G74" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H74" t="s">
+        <v>133</v>
+      </c>
+      <c r="I74">
+        <v>1</v>
+      </c>
+      <c r="J74">
+        <v>5</v>
+      </c>
+      <c r="K74" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB041 - Frequency of an Element
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E0F40E9-CD5B-40D8-9ED4-F95529500272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8257ADFE-70B1-4A15-B5A6-5952559E2439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="3360" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="229">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -735,6 +735,12 @@
   </si>
   <si>
     <t>Adajcent Element comparison</t>
+  </si>
+  <si>
+    <t>Count Frequency of Element in array</t>
+  </si>
+  <si>
+    <t>Couunting / Frequency Counting</t>
   </si>
 </sst>
 </file>
@@ -1254,7 +1260,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N74"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -3863,6 +3869,41 @@
       </c>
       <c r="K74" t="s">
         <v>226</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>36</v>
+      </c>
+      <c r="C75" t="s">
+        <v>227</v>
+      </c>
+      <c r="D75" t="s">
+        <v>76</v>
+      </c>
+      <c r="E75" t="s">
+        <v>114</v>
+      </c>
+      <c r="F75" t="s">
+        <v>77</v>
+      </c>
+      <c r="G75" s="2">
+        <v>46193</v>
+      </c>
+      <c r="H75" t="s">
+        <v>174</v>
+      </c>
+      <c r="I75">
+        <v>1</v>
+      </c>
+      <c r="J75">
+        <v>5</v>
+      </c>
+      <c r="K75" t="s">
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Completed Problems Array based on Leetcode and HackerRank
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8257ADFE-70B1-4A15-B5A6-5952559E2439}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FD3C47-F916-478B-B521-30F73543472C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="3360" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="2796" yWindow="3948" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="251">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -741,6 +741,72 @@
   </si>
   <si>
     <t>Couunting / Frequency Counting</t>
+  </si>
+  <si>
+    <t>Java 1D Array</t>
+  </si>
+  <si>
+    <t>Traversal</t>
+  </si>
+  <si>
+    <t>Java 1D Array (Part 2)</t>
+  </si>
+  <si>
+    <t>Linear Traversal, Conditions</t>
+  </si>
+  <si>
+    <t>Build Array from Permutation</t>
+  </si>
+  <si>
+    <t>Running Sum of 1D Array</t>
+  </si>
+  <si>
+    <t>12 min</t>
+  </si>
+  <si>
+    <t>Accumalator</t>
+  </si>
+  <si>
+    <t>Concatention of Array</t>
+  </si>
+  <si>
+    <t>Shuffle The array</t>
+  </si>
+  <si>
+    <t>index Manipulation</t>
+  </si>
+  <si>
+    <t>Richest Customer Wealth</t>
+  </si>
+  <si>
+    <t>2D Traversal, Maximum</t>
+  </si>
+  <si>
+    <t>Find the Highest Altitude</t>
+  </si>
+  <si>
+    <t>Running Sum, Maximum</t>
+  </si>
+  <si>
+    <t>Kids With Maximun Candies</t>
+  </si>
+  <si>
+    <t>18 min</t>
+  </si>
+  <si>
+    <t>Maximum Tracking</t>
+  </si>
+  <si>
+    <t>Max Consecutive Ones</t>
+  </si>
+  <si>
+    <t>Counting Pattern</t>
+  </si>
+  <si>
+    <t>Numbers smaller than current number</t>
+  </si>
+  <si>
+    <t>Traversal, Counting</t>
   </si>
 </sst>
 </file>
@@ -1260,7 +1326,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N86"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -1336,7 +1402,7 @@
         <v>77</v>
       </c>
       <c r="G2" s="2">
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="H2" t="s">
         <v>97</v>
@@ -1371,7 +1437,7 @@
         <v>77</v>
       </c>
       <c r="G3" s="2">
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="H3" t="s">
         <v>82</v>
@@ -1406,7 +1472,7 @@
         <v>77</v>
       </c>
       <c r="G4" s="2">
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="H4" t="s">
         <v>83</v>
@@ -1441,7 +1507,7 @@
         <v>77</v>
       </c>
       <c r="G5" s="2">
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="H5" t="s">
         <v>84</v>
@@ -1476,7 +1542,7 @@
         <v>77</v>
       </c>
       <c r="G6" s="2">
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="H6" t="s">
         <v>84</v>
@@ -1511,7 +1577,7 @@
         <v>77</v>
       </c>
       <c r="G7" s="2">
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="H7" t="s">
         <v>91</v>
@@ -1546,7 +1612,7 @@
         <v>77</v>
       </c>
       <c r="G8" s="2">
-        <v>46188</v>
+        <v>46212</v>
       </c>
       <c r="H8" t="s">
         <v>84</v>
@@ -1581,7 +1647,7 @@
         <v>77</v>
       </c>
       <c r="G9" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H9" t="s">
         <v>98</v>
@@ -1616,7 +1682,7 @@
         <v>77</v>
       </c>
       <c r="G10" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H10" t="s">
         <v>83</v>
@@ -1651,7 +1717,7 @@
         <v>77</v>
       </c>
       <c r="G11" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H11" t="s">
         <v>97</v>
@@ -1686,7 +1752,7 @@
         <v>77</v>
       </c>
       <c r="G12" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H12" t="s">
         <v>102</v>
@@ -1721,7 +1787,7 @@
         <v>77</v>
       </c>
       <c r="G13" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H13" t="s">
         <v>84</v>
@@ -1756,7 +1822,7 @@
         <v>77</v>
       </c>
       <c r="G14" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H14" t="s">
         <v>84</v>
@@ -1791,7 +1857,7 @@
         <v>77</v>
       </c>
       <c r="G15" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H15" t="s">
         <v>84</v>
@@ -1826,7 +1892,7 @@
         <v>77</v>
       </c>
       <c r="G16" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H16" t="s">
         <v>102</v>
@@ -1861,7 +1927,7 @@
         <v>77</v>
       </c>
       <c r="G17" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H17" t="s">
         <v>102</v>
@@ -1896,7 +1962,7 @@
         <v>77</v>
       </c>
       <c r="G18" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H18" t="s">
         <v>98</v>
@@ -1931,7 +1997,7 @@
         <v>77</v>
       </c>
       <c r="G19" s="2">
-        <v>46189</v>
+        <v>46213</v>
       </c>
       <c r="H19" t="s">
         <v>84</v>
@@ -1966,7 +2032,7 @@
         <v>77</v>
       </c>
       <c r="G20" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H20" t="s">
         <v>98</v>
@@ -2001,7 +2067,7 @@
         <v>77</v>
       </c>
       <c r="G21" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H21" t="s">
         <v>84</v>
@@ -2036,7 +2102,7 @@
         <v>77</v>
       </c>
       <c r="G22" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H22" t="s">
         <v>125</v>
@@ -2071,7 +2137,7 @@
         <v>77</v>
       </c>
       <c r="G23" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H23" t="s">
         <v>102</v>
@@ -2106,7 +2172,7 @@
         <v>77</v>
       </c>
       <c r="G24" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H24" t="s">
         <v>125</v>
@@ -2141,7 +2207,7 @@
         <v>77</v>
       </c>
       <c r="G25" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H25" t="s">
         <v>102</v>
@@ -2176,7 +2242,7 @@
         <v>77</v>
       </c>
       <c r="G26" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H26" t="s">
         <v>133</v>
@@ -2211,7 +2277,7 @@
         <v>77</v>
       </c>
       <c r="G27" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H27" t="s">
         <v>98</v>
@@ -2246,7 +2312,7 @@
         <v>77</v>
       </c>
       <c r="G28" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H28" t="s">
         <v>102</v>
@@ -2281,7 +2347,7 @@
         <v>77</v>
       </c>
       <c r="G29" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H29" t="s">
         <v>84</v>
@@ -2316,7 +2382,7 @@
         <v>77</v>
       </c>
       <c r="G30" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H30" t="s">
         <v>102</v>
@@ -2351,7 +2417,7 @@
         <v>77</v>
       </c>
       <c r="G31" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H31" t="s">
         <v>98</v>
@@ -2386,7 +2452,7 @@
         <v>77</v>
       </c>
       <c r="G32" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H32" t="s">
         <v>125</v>
@@ -2421,7 +2487,7 @@
         <v>77</v>
       </c>
       <c r="G33" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H33" t="s">
         <v>102</v>
@@ -2456,7 +2522,7 @@
         <v>77</v>
       </c>
       <c r="G34" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H34" t="s">
         <v>98</v>
@@ -2491,7 +2557,7 @@
         <v>77</v>
       </c>
       <c r="G35" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H35" t="s">
         <v>84</v>
@@ -2526,7 +2592,7 @@
         <v>77</v>
       </c>
       <c r="G36" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H36" t="s">
         <v>84</v>
@@ -2561,7 +2627,7 @@
         <v>77</v>
       </c>
       <c r="G37" s="2">
-        <v>46190</v>
+        <v>46214</v>
       </c>
       <c r="H37" t="s">
         <v>102</v>
@@ -2596,7 +2662,7 @@
         <v>77</v>
       </c>
       <c r="G38" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H38" t="s">
         <v>98</v>
@@ -2631,7 +2697,7 @@
         <v>77</v>
       </c>
       <c r="G39" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H39" t="s">
         <v>133</v>
@@ -2666,7 +2732,7 @@
         <v>77</v>
       </c>
       <c r="G40" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H40" t="s">
         <v>102</v>
@@ -2701,7 +2767,7 @@
         <v>77</v>
       </c>
       <c r="G41" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H41" t="s">
         <v>98</v>
@@ -2736,7 +2802,7 @@
         <v>77</v>
       </c>
       <c r="G42" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H42" t="s">
         <v>102</v>
@@ -2771,7 +2837,7 @@
         <v>77</v>
       </c>
       <c r="G43" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H43" t="s">
         <v>98</v>
@@ -2806,7 +2872,7 @@
         <v>77</v>
       </c>
       <c r="G44" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H44" t="s">
         <v>174</v>
@@ -2841,7 +2907,7 @@
         <v>77</v>
       </c>
       <c r="G45" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H45" t="s">
         <v>175</v>
@@ -2876,7 +2942,7 @@
         <v>77</v>
       </c>
       <c r="G46" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H46" t="s">
         <v>177</v>
@@ -2911,7 +2977,7 @@
         <v>77</v>
       </c>
       <c r="G47" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H47" t="s">
         <v>178</v>
@@ -2946,7 +3012,7 @@
         <v>77</v>
       </c>
       <c r="G48" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H48" t="s">
         <v>84</v>
@@ -2981,7 +3047,7 @@
         <v>77</v>
       </c>
       <c r="G49" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H49" t="s">
         <v>97</v>
@@ -3016,7 +3082,7 @@
         <v>77</v>
       </c>
       <c r="G50" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H50" t="s">
         <v>84</v>
@@ -3051,7 +3117,7 @@
         <v>77</v>
       </c>
       <c r="G51" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H51" t="s">
         <v>102</v>
@@ -3086,7 +3152,7 @@
         <v>77</v>
       </c>
       <c r="G52" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H52" t="s">
         <v>97</v>
@@ -3121,7 +3187,7 @@
         <v>77</v>
       </c>
       <c r="G53" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H53" t="s">
         <v>97</v>
@@ -3156,7 +3222,7 @@
         <v>77</v>
       </c>
       <c r="G54" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H54" t="s">
         <v>102</v>
@@ -3191,7 +3257,7 @@
         <v>77</v>
       </c>
       <c r="G55" s="2">
-        <v>46191</v>
+        <v>46215</v>
       </c>
       <c r="H55" t="s">
         <v>84</v>
@@ -3226,7 +3292,7 @@
         <v>77</v>
       </c>
       <c r="G56" s="2">
-        <v>46191</v>
+        <v>46216</v>
       </c>
       <c r="H56" t="s">
         <v>82</v>
@@ -3261,7 +3327,7 @@
         <v>77</v>
       </c>
       <c r="G57" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H57" t="s">
         <v>98</v>
@@ -3296,7 +3362,7 @@
         <v>77</v>
       </c>
       <c r="G58" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H58" t="s">
         <v>97</v>
@@ -3331,7 +3397,7 @@
         <v>77</v>
       </c>
       <c r="G59" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H59" t="s">
         <v>98</v>
@@ -3366,7 +3432,7 @@
         <v>77</v>
       </c>
       <c r="G60" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H60" t="s">
         <v>98</v>
@@ -3401,7 +3467,7 @@
         <v>77</v>
       </c>
       <c r="G61" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H61" t="s">
         <v>102</v>
@@ -3436,7 +3502,7 @@
         <v>77</v>
       </c>
       <c r="G62" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H62" t="s">
         <v>98</v>
@@ -3471,7 +3537,7 @@
         <v>77</v>
       </c>
       <c r="G63" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H63" t="s">
         <v>84</v>
@@ -3506,7 +3572,7 @@
         <v>77</v>
       </c>
       <c r="G64" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H64" t="s">
         <v>84</v>
@@ -3541,7 +3607,7 @@
         <v>77</v>
       </c>
       <c r="G65" s="2">
-        <v>46192</v>
+        <v>46216</v>
       </c>
       <c r="H65" t="s">
         <v>84</v>
@@ -3576,7 +3642,7 @@
         <v>77</v>
       </c>
       <c r="G66" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H66" t="s">
         <v>98</v>
@@ -3611,7 +3677,7 @@
         <v>77</v>
       </c>
       <c r="G67" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H67" t="s">
         <v>102</v>
@@ -3646,7 +3712,7 @@
         <v>77</v>
       </c>
       <c r="G68" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H68" t="s">
         <v>133</v>
@@ -3681,7 +3747,7 @@
         <v>77</v>
       </c>
       <c r="G69" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H69" t="s">
         <v>215</v>
@@ -3716,7 +3782,7 @@
         <v>77</v>
       </c>
       <c r="G70" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H70" t="s">
         <v>174</v>
@@ -3751,7 +3817,7 @@
         <v>77</v>
       </c>
       <c r="G71" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H71" t="s">
         <v>133</v>
@@ -3786,7 +3852,7 @@
         <v>77</v>
       </c>
       <c r="G72" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H72" t="s">
         <v>125</v>
@@ -3821,7 +3887,7 @@
         <v>77</v>
       </c>
       <c r="G73" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H73" t="s">
         <v>102</v>
@@ -3856,7 +3922,7 @@
         <v>77</v>
       </c>
       <c r="G74" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H74" t="s">
         <v>133</v>
@@ -3891,7 +3957,7 @@
         <v>77</v>
       </c>
       <c r="G75" s="2">
-        <v>46193</v>
+        <v>46217</v>
       </c>
       <c r="H75" t="s">
         <v>174</v>
@@ -3904,6 +3970,391 @@
       </c>
       <c r="K75" t="s">
         <v>228</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>36</v>
+      </c>
+      <c r="C76" t="s">
+        <v>229</v>
+      </c>
+      <c r="D76" t="s">
+        <v>81</v>
+      </c>
+      <c r="E76" t="s">
+        <v>114</v>
+      </c>
+      <c r="F76" t="s">
+        <v>77</v>
+      </c>
+      <c r="G76" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H76" t="s">
+        <v>133</v>
+      </c>
+      <c r="I76">
+        <v>1</v>
+      </c>
+      <c r="J76">
+        <v>5</v>
+      </c>
+      <c r="K76" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>36</v>
+      </c>
+      <c r="C77" t="s">
+        <v>231</v>
+      </c>
+      <c r="D77" t="s">
+        <v>81</v>
+      </c>
+      <c r="E77" t="s">
+        <v>114</v>
+      </c>
+      <c r="F77" t="s">
+        <v>77</v>
+      </c>
+      <c r="G77" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H77" t="s">
+        <v>174</v>
+      </c>
+      <c r="I77">
+        <v>1</v>
+      </c>
+      <c r="J77">
+        <v>5</v>
+      </c>
+      <c r="K77" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>36</v>
+      </c>
+      <c r="C78" t="s">
+        <v>233</v>
+      </c>
+      <c r="D78" t="s">
+        <v>145</v>
+      </c>
+      <c r="E78" t="s">
+        <v>114</v>
+      </c>
+      <c r="F78" t="s">
+        <v>77</v>
+      </c>
+      <c r="G78" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H78" t="s">
+        <v>175</v>
+      </c>
+      <c r="I78">
+        <v>1</v>
+      </c>
+      <c r="J78">
+        <v>5</v>
+      </c>
+      <c r="K78" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>36</v>
+      </c>
+      <c r="C79" t="s">
+        <v>234</v>
+      </c>
+      <c r="D79" t="s">
+        <v>145</v>
+      </c>
+      <c r="E79" t="s">
+        <v>114</v>
+      </c>
+      <c r="F79" t="s">
+        <v>77</v>
+      </c>
+      <c r="G79" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H79" t="s">
+        <v>235</v>
+      </c>
+      <c r="I79">
+        <v>1</v>
+      </c>
+      <c r="J79">
+        <v>5</v>
+      </c>
+      <c r="K79" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>36</v>
+      </c>
+      <c r="C80" t="s">
+        <v>237</v>
+      </c>
+      <c r="D80" t="s">
+        <v>145</v>
+      </c>
+      <c r="E80" t="s">
+        <v>114</v>
+      </c>
+      <c r="F80" t="s">
+        <v>77</v>
+      </c>
+      <c r="G80" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H80" t="s">
+        <v>175</v>
+      </c>
+      <c r="I80">
+        <v>1</v>
+      </c>
+      <c r="J80">
+        <v>5</v>
+      </c>
+      <c r="K80" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>36</v>
+      </c>
+      <c r="C81" t="s">
+        <v>238</v>
+      </c>
+      <c r="D81" t="s">
+        <v>145</v>
+      </c>
+      <c r="E81" t="s">
+        <v>114</v>
+      </c>
+      <c r="F81" t="s">
+        <v>77</v>
+      </c>
+      <c r="G81" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H81" t="s">
+        <v>174</v>
+      </c>
+      <c r="I81">
+        <v>1</v>
+      </c>
+      <c r="J81">
+        <v>5</v>
+      </c>
+      <c r="K81" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>36</v>
+      </c>
+      <c r="C82" t="s">
+        <v>240</v>
+      </c>
+      <c r="D82" t="s">
+        <v>145</v>
+      </c>
+      <c r="E82" t="s">
+        <v>114</v>
+      </c>
+      <c r="F82" t="s">
+        <v>77</v>
+      </c>
+      <c r="G82" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H82" t="s">
+        <v>175</v>
+      </c>
+      <c r="I82">
+        <v>1</v>
+      </c>
+      <c r="J82">
+        <v>5</v>
+      </c>
+      <c r="K82" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>36</v>
+      </c>
+      <c r="C83" t="s">
+        <v>242</v>
+      </c>
+      <c r="D83" t="s">
+        <v>145</v>
+      </c>
+      <c r="E83" t="s">
+        <v>114</v>
+      </c>
+      <c r="F83" t="s">
+        <v>77</v>
+      </c>
+      <c r="G83" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H83" t="s">
+        <v>235</v>
+      </c>
+      <c r="I83">
+        <v>1</v>
+      </c>
+      <c r="J83">
+        <v>5</v>
+      </c>
+      <c r="K83" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>36</v>
+      </c>
+      <c r="C84" t="s">
+        <v>244</v>
+      </c>
+      <c r="D84" t="s">
+        <v>145</v>
+      </c>
+      <c r="E84" t="s">
+        <v>5</v>
+      </c>
+      <c r="F84" t="s">
+        <v>77</v>
+      </c>
+      <c r="G84" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H84" t="s">
+        <v>245</v>
+      </c>
+      <c r="I84">
+        <v>1</v>
+      </c>
+      <c r="J84">
+        <v>5</v>
+      </c>
+      <c r="K84" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>36</v>
+      </c>
+      <c r="C85" t="s">
+        <v>247</v>
+      </c>
+      <c r="D85" t="s">
+        <v>145</v>
+      </c>
+      <c r="E85" t="s">
+        <v>4</v>
+      </c>
+      <c r="F85" t="s">
+        <v>77</v>
+      </c>
+      <c r="G85" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H85" t="s">
+        <v>133</v>
+      </c>
+      <c r="I85">
+        <v>1</v>
+      </c>
+      <c r="J85">
+        <v>5</v>
+      </c>
+      <c r="K85" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>36</v>
+      </c>
+      <c r="C86" t="s">
+        <v>249</v>
+      </c>
+      <c r="D86" t="s">
+        <v>145</v>
+      </c>
+      <c r="E86" t="s">
+        <v>4</v>
+      </c>
+      <c r="F86" t="s">
+        <v>77</v>
+      </c>
+      <c r="G86" s="2">
+        <v>46217</v>
+      </c>
+      <c r="H86" t="s">
+        <v>175</v>
+      </c>
+      <c r="I86">
+        <v>1</v>
+      </c>
+      <c r="J86">
+        <v>5</v>
+      </c>
+      <c r="K86" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB042 - String Input and Output
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7FD3C47-F916-478B-B521-30F73543472C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84783D6A-90E9-433E-8A40-008FFBB71134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2796" yWindow="3948" windowWidth="19296" windowHeight="8880" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -807,6 +807,72 @@
   </si>
   <si>
     <t>Traversal, Counting</t>
+  </si>
+  <si>
+    <t>Java ArrayList</t>
+  </si>
+  <si>
+    <t>Dynamic Array</t>
+  </si>
+  <si>
+    <t>Java SubArray</t>
+  </si>
+  <si>
+    <t>Nested Loops, Accumalator</t>
+  </si>
+  <si>
+    <t>2D Array</t>
+  </si>
+  <si>
+    <t>Java 2D Array</t>
+  </si>
+  <si>
+    <t>String Input and Output</t>
+  </si>
+  <si>
+    <t>String Length</t>
+  </si>
+  <si>
+    <t>Reverse a String</t>
+  </si>
+  <si>
+    <t>Palindrome String</t>
+  </si>
+  <si>
+    <t>Count Vowels and Consonants</t>
+  </si>
+  <si>
+    <t>Count Words</t>
+  </si>
+  <si>
+    <t>Count Characters</t>
+  </si>
+  <si>
+    <t>Toggle Case</t>
+  </si>
+  <si>
+    <t>Remove Spaces</t>
+  </si>
+  <si>
+    <t>Check Anagram</t>
+  </si>
+  <si>
+    <t>Built-in Methods</t>
+  </si>
+  <si>
+    <t>Multiple Accumulators</t>
+  </si>
+  <si>
+    <t>Traversal, Conditions</t>
+  </si>
+  <si>
+    <t>Frequency Counting</t>
+  </si>
+  <si>
+    <t>Character Manipulation</t>
+  </si>
+  <si>
+    <t>String Building</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1392,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1910367-E57A-4A31-95CF-86632858D800}">
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N100"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.77734375" customWidth="1"/>
@@ -4355,6 +4421,334 @@
       </c>
       <c r="K86" t="s">
         <v>250</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>36</v>
+      </c>
+      <c r="C87" t="s">
+        <v>251</v>
+      </c>
+      <c r="D87" t="s">
+        <v>81</v>
+      </c>
+      <c r="E87" t="s">
+        <v>114</v>
+      </c>
+      <c r="F87" t="s">
+        <v>77</v>
+      </c>
+      <c r="G87" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H87" t="s">
+        <v>175</v>
+      </c>
+      <c r="I87">
+        <v>1</v>
+      </c>
+      <c r="J87">
+        <v>5</v>
+      </c>
+      <c r="K87" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A88">
+        <v>87</v>
+      </c>
+      <c r="B88" t="s">
+        <v>36</v>
+      </c>
+      <c r="C88" t="s">
+        <v>253</v>
+      </c>
+      <c r="D88" t="s">
+        <v>81</v>
+      </c>
+      <c r="E88" t="s">
+        <v>114</v>
+      </c>
+      <c r="F88" t="s">
+        <v>77</v>
+      </c>
+      <c r="G88" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H88" t="s">
+        <v>174</v>
+      </c>
+      <c r="I88">
+        <v>1</v>
+      </c>
+      <c r="J88">
+        <v>5</v>
+      </c>
+      <c r="K88" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A89">
+        <v>88</v>
+      </c>
+      <c r="B89" t="s">
+        <v>36</v>
+      </c>
+      <c r="C89" t="s">
+        <v>256</v>
+      </c>
+      <c r="D89" t="s">
+        <v>81</v>
+      </c>
+      <c r="E89" t="s">
+        <v>114</v>
+      </c>
+      <c r="F89" t="s">
+        <v>77</v>
+      </c>
+      <c r="G89" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H89" t="s">
+        <v>177</v>
+      </c>
+      <c r="I89">
+        <v>1</v>
+      </c>
+      <c r="J89">
+        <v>5</v>
+      </c>
+      <c r="K89" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A90">
+        <v>89</v>
+      </c>
+      <c r="B90" t="s">
+        <v>39</v>
+      </c>
+      <c r="C90" t="s">
+        <v>257</v>
+      </c>
+      <c r="D90" t="s">
+        <v>76</v>
+      </c>
+      <c r="E90" t="s">
+        <v>4</v>
+      </c>
+      <c r="F90" t="s">
+        <v>77</v>
+      </c>
+      <c r="G90" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H90" t="s">
+        <v>102</v>
+      </c>
+      <c r="I90">
+        <v>1</v>
+      </c>
+      <c r="J90">
+        <v>5</v>
+      </c>
+      <c r="K90" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A91">
+        <v>90</v>
+      </c>
+      <c r="B91" t="s">
+        <v>39</v>
+      </c>
+      <c r="C91" t="s">
+        <v>258</v>
+      </c>
+      <c r="D91" t="s">
+        <v>76</v>
+      </c>
+      <c r="E91" t="s">
+        <v>4</v>
+      </c>
+      <c r="K91" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A92">
+        <v>91</v>
+      </c>
+      <c r="B92" t="s">
+        <v>39</v>
+      </c>
+      <c r="C92" t="s">
+        <v>259</v>
+      </c>
+      <c r="D92" t="s">
+        <v>76</v>
+      </c>
+      <c r="E92" t="s">
+        <v>114</v>
+      </c>
+      <c r="K92" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A93">
+        <v>92</v>
+      </c>
+      <c r="B93" t="s">
+        <v>39</v>
+      </c>
+      <c r="C93" t="s">
+        <v>260</v>
+      </c>
+      <c r="D93" t="s">
+        <v>76</v>
+      </c>
+      <c r="E93" t="s">
+        <v>114</v>
+      </c>
+      <c r="K93" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94">
+        <v>93</v>
+      </c>
+      <c r="B94" t="s">
+        <v>39</v>
+      </c>
+      <c r="C94" t="s">
+        <v>261</v>
+      </c>
+      <c r="D94" t="s">
+        <v>76</v>
+      </c>
+      <c r="E94" t="s">
+        <v>114</v>
+      </c>
+      <c r="K94" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95">
+        <v>94</v>
+      </c>
+      <c r="B95" t="s">
+        <v>39</v>
+      </c>
+      <c r="C95" t="s">
+        <v>262</v>
+      </c>
+      <c r="D95" t="s">
+        <v>76</v>
+      </c>
+      <c r="E95" t="s">
+        <v>114</v>
+      </c>
+      <c r="K95" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A96">
+        <v>95</v>
+      </c>
+      <c r="B96" t="s">
+        <v>39</v>
+      </c>
+      <c r="C96" t="s">
+        <v>263</v>
+      </c>
+      <c r="D96" t="s">
+        <v>76</v>
+      </c>
+      <c r="E96" t="s">
+        <v>114</v>
+      </c>
+      <c r="K96" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A97">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>39</v>
+      </c>
+      <c r="C97" t="s">
+        <v>264</v>
+      </c>
+      <c r="D97" t="s">
+        <v>76</v>
+      </c>
+      <c r="E97" t="s">
+        <v>114</v>
+      </c>
+      <c r="K97" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A98">
+        <v>97</v>
+      </c>
+      <c r="B98" t="s">
+        <v>39</v>
+      </c>
+      <c r="C98" t="s">
+        <v>265</v>
+      </c>
+      <c r="D98" t="s">
+        <v>76</v>
+      </c>
+      <c r="E98" t="s">
+        <v>114</v>
+      </c>
+      <c r="K98" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A99">
+        <v>98</v>
+      </c>
+      <c r="B99" t="s">
+        <v>39</v>
+      </c>
+      <c r="C99" t="s">
+        <v>266</v>
+      </c>
+      <c r="D99" t="s">
+        <v>76</v>
+      </c>
+      <c r="E99" t="s">
+        <v>5</v>
+      </c>
+      <c r="K99" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A100">
+        <v>99</v>
+      </c>
+      <c r="B100" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solve PB043 - String Length
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84783D6A-90E9-433E-8A40-008FFBB71134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99EAABA2-90C3-488B-8A8C-A16F93172F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="770" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4579,6 +4579,21 @@
       <c r="E91" t="s">
         <v>4</v>
       </c>
+      <c r="F91" t="s">
+        <v>77</v>
+      </c>
+      <c r="G91" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H91" t="s">
+        <v>102</v>
+      </c>
+      <c r="I91">
+        <v>1</v>
+      </c>
+      <c r="J91">
+        <v>5</v>
+      </c>
       <c r="K91" t="s">
         <v>267</v>
       </c>

</xml_diff>

<commit_message>
Solve PB044 - Reverse String
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99EAABA2-90C3-488B-8A8C-A16F93172F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0E70D6-7009-4F54-84B8-3E134A97A08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="772" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4614,6 +4614,21 @@
       <c r="E92" t="s">
         <v>114</v>
       </c>
+      <c r="F92" t="s">
+        <v>77</v>
+      </c>
+      <c r="G92" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H92" t="s">
+        <v>133</v>
+      </c>
+      <c r="I92">
+        <v>1</v>
+      </c>
+      <c r="J92">
+        <v>5</v>
+      </c>
       <c r="K92" t="s">
         <v>220</v>
       </c>

</xml_diff>

<commit_message>
Solve PB045 - Palindrome String
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0E70D6-7009-4F54-84B8-3E134A97A08E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E228A5EA-118F-4FAD-9247-95A6F577A274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4649,6 +4649,21 @@
       <c r="E93" t="s">
         <v>114</v>
       </c>
+      <c r="F93" t="s">
+        <v>77</v>
+      </c>
+      <c r="G93" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H93" t="s">
+        <v>174</v>
+      </c>
+      <c r="I93">
+        <v>1</v>
+      </c>
+      <c r="J93">
+        <v>5</v>
+      </c>
       <c r="K93" t="s">
         <v>220</v>
       </c>

</xml_diff>

<commit_message>
Solve PB046 - Count Vowels and Consonants
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E228A5EA-118F-4FAD-9247-95A6F577A274}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBDE6AED-467B-49D4-B564-0CDFAB0A148B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4684,6 +4684,21 @@
       <c r="E94" t="s">
         <v>114</v>
       </c>
+      <c r="F94" t="s">
+        <v>77</v>
+      </c>
+      <c r="G94" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H94" t="s">
+        <v>174</v>
+      </c>
+      <c r="I94">
+        <v>1</v>
+      </c>
+      <c r="J94">
+        <v>5</v>
+      </c>
       <c r="K94" t="s">
         <v>268</v>
       </c>

</xml_diff>

<commit_message>
Solve PB047 - Count Words
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBDE6AED-467B-49D4-B564-0CDFAB0A148B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20DA868-5025-469A-BDEA-583C155B4802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="778" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4719,6 +4719,21 @@
       <c r="E95" t="s">
         <v>114</v>
       </c>
+      <c r="F95" t="s">
+        <v>77</v>
+      </c>
+      <c r="G95" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H95" t="s">
+        <v>175</v>
+      </c>
+      <c r="I95">
+        <v>1</v>
+      </c>
+      <c r="J95">
+        <v>5</v>
+      </c>
       <c r="K95" t="s">
         <v>269</v>
       </c>

</xml_diff>

<commit_message>
Solve PB048 - Character Frequency
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C20DA868-5025-469A-BDEA-583C155B4802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D19818-993B-439F-BB3A-DF82773ED35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="780" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4754,6 +4754,21 @@
       <c r="E96" t="s">
         <v>114</v>
       </c>
+      <c r="F96" t="s">
+        <v>77</v>
+      </c>
+      <c r="G96" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H96" t="s">
+        <v>175</v>
+      </c>
+      <c r="I96">
+        <v>1</v>
+      </c>
+      <c r="J96">
+        <v>5</v>
+      </c>
       <c r="K96" t="s">
         <v>270</v>
       </c>

</xml_diff>

<commit_message>
Solve PB049 - Toggle Case
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01D19818-993B-439F-BB3A-DF82773ED35B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEC3A94-41BF-4972-B391-9B8F86720A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4789,6 +4789,21 @@
       <c r="E97" t="s">
         <v>114</v>
       </c>
+      <c r="F97" t="s">
+        <v>77</v>
+      </c>
+      <c r="G97" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H97" t="s">
+        <v>175</v>
+      </c>
+      <c r="I97">
+        <v>1</v>
+      </c>
+      <c r="J97">
+        <v>5</v>
+      </c>
       <c r="K97" t="s">
         <v>271</v>
       </c>

</xml_diff>

<commit_message>
Solve PB050 - Remove Spaces
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEC3A94-41BF-4972-B391-9B8F86720A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD40D92-494D-46FB-BC95-9566A29D52B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="784" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4822,7 +4822,22 @@
         <v>76</v>
       </c>
       <c r="E98" t="s">
-        <v>114</v>
+        <v>4</v>
+      </c>
+      <c r="F98" t="s">
+        <v>77</v>
+      </c>
+      <c r="G98" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H98" t="s">
+        <v>174</v>
+      </c>
+      <c r="I98">
+        <v>1</v>
+      </c>
+      <c r="J98">
+        <v>5</v>
       </c>
       <c r="K98" t="s">
         <v>272</v>

</xml_diff>

<commit_message>
Solve PB051 - Check Anagram
</commit_message>
<xml_diff>
--- a/Java_DSA_Mastery_Tracker.xlsx
+++ b/Java_DSA_Mastery_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\Java-DSA-Mastery\java-dsa-mastery\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DDD40D92-494D-46FB-BC95-9566A29D52B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56F33EC7-089E-453E-98F7-C0627AD503DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="1" xr2:uid="{74AE5DD4-9E62-4679-B045-983C6EEEAE70}"/>
   </bookViews>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="273">
   <si>
     <t>JAVA DSA MASTERY DASHBOARD</t>
   </si>
@@ -4859,6 +4859,21 @@
       <c r="E99" t="s">
         <v>5</v>
       </c>
+      <c r="F99" t="s">
+        <v>77</v>
+      </c>
+      <c r="G99" s="2">
+        <v>46188</v>
+      </c>
+      <c r="H99" t="s">
+        <v>177</v>
+      </c>
+      <c r="I99">
+        <v>1</v>
+      </c>
+      <c r="J99">
+        <v>5</v>
+      </c>
       <c r="K99" t="s">
         <v>248</v>
       </c>

</xml_diff>